<commit_message>
feat: improve interview authoring and student usability
</commit_message>
<xml_diff>
--- a/grade34/templates/class-roster-template.xlsx
+++ b/grade34/templates/class-roster-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="名簿入力" sheetId="1" r:id="Rd6bfcc32183241ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R1fab3671a01c4bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="名簿入力" sheetId="1" r:id="R6d1db9180f504b47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Ra12b08dbbdfe45f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -664,46 +664,48 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>出席番号と、活動で使う名前の表記だけ入力してください。</x:v>
+        <x:v>出席番号は必須です。名前は使いたい表記だけ入力し、すべて空欄でも使えます。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>ひらがなの名前のみ：A列（出席番号）とE列（名前・ひらがな）を入力します。</x:v>
+        <x:v>番号だけで使う場合：A列（出席番号）のみ入力し、A列のみコピーしてください。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>英語の名前のみ：A列（出席番号）とG列（名前・英語）を入力します。</x:v>
+        <x:v>ひらがなの名前のみ：A列（出席番号）とE列（名前・ひらがな）を入力します。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>使わない表記の列は空欄でかまいません。出席番号は重複させないでください。</x:v>
+        <x:v>英語の名前のみ：A列（出席番号）とG列（名前・英語）を入力します。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>入力後は、名簿入力シートのA列からG列まで、空欄も含めてコピーします。</x:v>
+        <x:v>使わない表記の列は空欄でかまいません。出席番号は重複させないでください。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="9" t="str">
-        <x:v>クラス設定の「名簿を貼り付け」に貼り付け、「名簿を確認」→「名簿を保存」。</x:v>
+        <x:v>名前も使う場合：名簿入力シートのA列からG列まで、空欄も含めてコピーします。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="9" t="str">
-        <x:v>見出し行も一緒にコピーできます。35人分の空欄を用意しています。</x:v>
+        <x:v>クラス設定の「名簿を貼り付け」に貼り付け、「名簿を確認」→「名簿を保存」。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="9" t="str">
+        <x:v>見出し行も一緒にコピーできます。35人分の空欄を用意しています。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="9" t="str">
         <x:v>Excelで編集できます。Googleスプレッドシートへ読み込んで使うこともできます。</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="9"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="9"/>

</xml_diff>